<commit_message>
Update CyberShield NIC API Schema Excel file with latest changes.
</commit_message>
<xml_diff>
--- a/docs/CyberShield_NIC_API_Schema.xlsx
+++ b/docs/CyberShield_NIC_API_Schema.xlsx
@@ -9,8 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REST Endpoints" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WebSocket Events" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums &amp; Status Codes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Headers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagination" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Error Responses" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query Parameters" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Practices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WebSocket Events" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums &amp; Status Codes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +65,62 @@
       <name val="Consolas"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="001F4E78"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="0044546A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +143,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2933"/>
         <bgColor rgb="001F2933"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00366092"/>
+        <bgColor rgb="00366092"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+        <bgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0044546A"/>
+        <bgColor rgb="0044546A"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +221,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1006,7 +1119,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>query: severity, status, from, to, limit, offset</t>
+          <t>query: *limit, *offset, severity, status, from, to</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1090,7 +1203,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>{ note? }</t>
+          <t>{ note? (string, optional) }</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1132,12 +1245,12 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>query: anomaly_id, campaign, limit</t>
+          <t>query: *limit, *offset, anomaly_id, campaign</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>{ items: [ { attribution_id, anomaly_id, mitre_technique_id, mitre_tactic, matched_campaign, confidence, created_at } ], total }</t>
+          <t>{ items: [ { attribution_id, anomaly_id, mitre_technique_id, mitre_tactic, matched_campaign, confidence, created_at } ], total, limit, offset }</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1300,12 +1413,12 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>query: min_risk_score, status, limit, offset</t>
+          <t>query: *limit, *offset, min_risk_score, status</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>{ items: [ { vulnerability_id, cve_id, asset_id, risk_score, exploitability, description, status } ], total }</t>
+          <t>{ items: [ { vulnerability_id, cve_id, asset_id, risk_score, exploitability, description, status } ], total, limit, offset }</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1426,12 +1539,12 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>query: status, limit, offset</t>
+          <t>query: *limit, *offset, status</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>{ items: [ { action_id, anomaly_id, action_type, blast_radius, confidence, status, created_at } ], total }</t>
+          <t>{ items: [ { action_id, anomaly_id, action_type, blast_radius, confidence, status, created_at } ], total, limit, offset }</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1510,7 +1623,7 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>{ note? }</t>
+          <t>{ note? (string, optional) }</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -1636,12 +1749,12 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>query: type, segment, limit, offset</t>
+          <t>query: *limit, *offset, type, segment</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>{ items: [ { asset_id, name, type, segment, criticality, ip_address } ], total }</t>
+          <t>{ items: [ { asset_id, name, type, segment, criticality, ip_address } ], total, limit, offset }</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1720,12 +1833,12 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>query: agent, from, to, limit, offset</t>
+          <t>query: *limit, *offset, agent, from, to</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>{ items: [ { audit_id, agent, action_summary, reasoning, confidence, timestamp } ], total }</t>
+          <t>{ items: [ { audit_id, agent, action_summary, reasoning, confidence, timestamp } ], total, limit, offset }</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1762,12 +1875,12 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>query: since</t>
+          <t>query: *limit, *offset, since</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>{ items: [ { cve_id, published_at, severity, description } ], total }</t>
+          <t>{ items: [ { cve_id, published_at, severity, description } ], total, limit, offset }</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1791,6 +1904,1718 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Header Name</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Always Present</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Example Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Content-Type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Response content type</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>application/json; charset=utf-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>X-Request-ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>String (UUID)</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Unique request identifier for tracing</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>f47ac10b-58cc-4372-a567-0e02b2c3d479</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>X-RateLimit-Limit</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Maximum requests allowed in window</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>X-RateLimit-Remaining</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Requests remaining in current window</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>X-RateLimit-Reset</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Integer (Unix timestamp)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Epoch time when rate limit resets</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>1625097600</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Retry-After</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Integer (seconds)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>On 429</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Seconds to wait before retrying</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Cache-Control</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Selective</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Cache directives for GET requests</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>max-age=300, public</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>ETag</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Selective</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Entity tag for cache validation</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>"abc123def456"</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Pagination Specification</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All list endpoints accept and return pagination parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Query Parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Number of items per page (max 100, default 20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Zero-indexed offset for pagination (default 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Response Fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Array of resources matching query</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>[{...}, {...}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Total count of items (ignoring limit/offset)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Limit used in request</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Offset used in request</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>GET /api/v1/anomalies?limit=10&amp;offset=0     -&gt; returns items 0-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>GET /api/v1/anomalies?limit=10&amp;offset=10    -&gt; returns items 10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>GET /api/v1/anomalies?limit=10&amp;offset=20    -&gt; returns items 20-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Response: { items: [...], total: 150, limit: 10, offset: 0 }</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Error Response Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>HTTP Code</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Error Code</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>When It Occurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>BAD_REQUEST</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Invalid query parameters or request body</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Malformed limit/offset, invalid severity enum, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="n">
+        <v>401</v>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>UNAUTHORIZED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Missing or invalid authorization token</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bearer token missing, expired, or invalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="n">
+        <v>403</v>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>User role insufficient for this operation</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Analyst trying to access admin-only endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="n">
+        <v>404</v>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Resource with given ID does not exist</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GET /anomalies/invalid-id returns 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="n">
+        <v>409</v>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Action cannot be performed due to current state</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Approving an already-executed action</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="n">
+        <v>422</v>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Request body fails schema validation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Required field missing or wrong type</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="n">
+        <v>429</v>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>RATE_LIMITED</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Too many requests in rate limit window</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Exceeded 1000 req/minute limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>INTERNAL_ERROR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Unhandled server-side error</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Backend service crashed or query failed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Query Parameter Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Description/Values</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>/anomalies</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>/anomalies</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>/anomalies</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Filter: low | medium | high | critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>/anomalies</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Filter: new | investigating | acknowledged | contained | false_positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>/anomalies</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ISO8601</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Filter: start date (e.g., 2024-01-01T00:00:00Z)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>/anomalies</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ISO8601</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Filter: end date (e.g., 2024-01-31T23:59:59Z)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>/attributions</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>/attributions</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>/attributions</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>anomaly_id</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Filter: attribution for specific anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>/attributions</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>campaign</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Filter: by campaign name</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>/vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>/vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>/vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>min_risk_score</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Filter: minimum risk score (0-100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>/vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Filter: open | in_progress | patched | deferred | accepted_risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>/actions</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>/actions</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>/actions</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Filter: pending | approved | escalated | rejected | executed | failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>/assets</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>/assets</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>/assets</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Filter: server | workstation | network_device | ot_device | database</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>/assets</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Filter: network segment name</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>/audit-trail</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>/audit-trail</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>/audit-trail</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Filter: human | ml_engine | orchestrator | user</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>/audit-trail</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ISO8601</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Filter: start date</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>/audit-trail</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ISO8601</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Filter: end date</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>/cve-feed</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>limit</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Max items per page (default: 20, max: 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>/cve-feed</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Pagination offset (default: 0, zero-indexed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>/cve-feed</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>since</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ISO8601</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Filter: CVEs published since this date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>API Best Practices &amp; Implementation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>1. Always include X-Request-ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Every response includes X-Request-ID header for request tracing and debugging</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>2. Implement exponential backoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>On 429 (Rate Limited): wait Retry-After seconds, then exponential backoff (1s, 2s, 4s, ...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>3. Parse X-RateLimit headers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Check X-RateLimit-Remaining before each request to avoid hitting limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>4. Handle pagination properly</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>Always check `total` field to determine if more pages exist beyond current offset</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>5. Cache GET responses</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Use Cache-Control and ETag headers to reduce load and improve performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>6. Validate enum values</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Never send unknown enum values (e.g., severity=EXTREME). See Enums sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>7. Use ISO8601 timestamps</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>All timestamps are UTC. Parse as ISO8601, store as UTC, display in user timezone</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>8. Implement circuit breaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>If 3+ consecutive 500 errors, stop retrying for 30 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>9. Batch list requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Request limit=100 (max) to minimize total API calls for bulk operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>10. Add request IDs to logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Log X-Request-ID with every request for correlation with server logs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2004,7 +3829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>